<commit_message>
feat: implement delivery spec detection and safe excel merging to prevent corruption
</commit_message>
<xml_diff>
--- a/iatf_system/lib/excel_templates/apqp_plan_report_modified.xlsx
+++ b/iatf_system/lib/excel_templates/apqp_plan_report_modified.xlsx
@@ -2292,7 +2292,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac">
-  <dimension ref="A1:U65"/>
+  <dimension ref="A1:U70"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="2" width="4.09765625" style="1" customWidth="1"/>
@@ -3081,77 +3081,64 @@
       <c r="B30" s="16"/>
       <c r="C30" s="16"/>
       <c r="D30" s="17"/>
-      <c r="E30" s="21" t="s">
-        <v>99</v>
-      </c>
-      <c r="F30" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="G30" s="30"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="30"/>
-      <c r="K30" s="30"/>
-      <c r="L30" s="31"/>
-      <c r="M30" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="N30" s="30"/>
-      <c r="O30" s="30"/>
-      <c r="P30" s="30"/>
-      <c r="Q30" s="30"/>
-      <c r="R30" s="30"/>
-      <c r="S30" s="30"/>
-      <c r="T30" s="31"/>
-    </row>
-    <row r="31" spans="1:21" customFormat="false">
+      <c r="E30" s="21"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="I30" s="22"/>
+      <c r="J30" s="22"/>
+      <c r="K30" s="22"/>
+      <c r="L30" s="23"/>
+      <c r="M30" s="40" t="str">
+        <v>報告書名：#{?dr_setsubi_filename_3}</v>
+      </c>
+      <c r="N30" s="41"/>
+      <c r="O30" s="41"/>
+      <c r="P30" s="41"/>
+      <c r="Q30" s="41"/>
+      <c r="R30" s="41"/>
+      <c r="S30" s="41"/>
+      <c r="T30" s="42"/>
+    </row>
+    <row r="31" spans="1:20" customFormat="false">
       <c r="A31" s="12"/>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="F31" s="82" t="s">
-        <v>59</v>
-      </c>
-      <c r="G31" s="82"/>
-      <c r="H31" s="82"/>
-      <c r="I31" s="82"/>
-      <c r="J31" s="82"/>
-      <c r="K31" s="82"/>
-      <c r="L31" s="83"/>
-      <c r="M31" s="131"/>
-      <c r="N31" s="132"/>
-      <c r="O31" s="132"/>
-      <c r="P31" s="132"/>
-      <c r="Q31" s="132"/>
-      <c r="R31" s="132"/>
-      <c r="S31" s="132"/>
-      <c r="T31" s="133"/>
-      <c r="U31" s="13"/>
-    </row>
-    <row r="32" spans="1:20" customFormat="false" ht="33" customHeight="1">
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="I31" s="22"/>
+      <c r="J31" s="22"/>
+      <c r="K31" s="22"/>
+      <c r="L31" s="23"/>
+      <c r="M31" s="40" t="str">
+        <v>報告書名：#{?dr_setsubi_filename_4}</v>
+      </c>
+      <c r="N31" s="41"/>
+      <c r="O31" s="41"/>
+      <c r="P31" s="41"/>
+      <c r="Q31" s="41"/>
+      <c r="R31" s="41"/>
+      <c r="S31" s="41"/>
+      <c r="T31" s="42"/>
+    </row>
+    <row r="32" spans="1:20" customFormat="false">
       <c r="A32" s="12"/>
-      <c r="B32" s="102" t="s">
-        <v>25</v>
-      </c>
-      <c r="C32" s="102"/>
-      <c r="D32" s="102"/>
-      <c r="E32" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="F32" s="30" t="s">
-        <v>40</v>
-      </c>
-      <c r="G32" s="30"/>
-      <c r="H32" s="30"/>
-      <c r="I32" s="30"/>
-      <c r="J32" s="30"/>
-      <c r="K32" s="30"/>
-      <c r="L32" s="31"/>
-      <c r="M32" s="40" t="s">
-        <v>81</v>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22"/>
+      <c r="J32" s="22"/>
+      <c r="K32" s="22"/>
+      <c r="L32" s="23"/>
+      <c r="M32" s="40" t="str">
+        <v>報告書名：#{?dr_setsubi_filename_5}</v>
       </c>
       <c r="N32" s="41"/>
       <c r="O32" s="41"/>
@@ -3161,156 +3148,149 @@
       <c r="S32" s="41"/>
       <c r="T32" s="42"/>
     </row>
-    <row r="33" spans="1:20" customFormat="false" ht="33" customHeight="1">
+    <row r="33" spans="1:20" customFormat="false">
       <c r="A33" s="12"/>
-      <c r="B33" s="15"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="F33" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
-      <c r="I33" s="30"/>
-      <c r="J33" s="30"/>
-      <c r="K33" s="30"/>
-      <c r="L33" s="31"/>
-      <c r="M33" s="32" t="s">
-        <v>77</v>
-      </c>
-      <c r="N33" s="33"/>
-      <c r="O33" s="33"/>
-      <c r="P33" s="33"/>
-      <c r="Q33" s="33"/>
-      <c r="R33" s="33"/>
-      <c r="S33" s="33"/>
-      <c r="T33" s="34"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="I33" s="22"/>
+      <c r="J33" s="22"/>
+      <c r="K33" s="22"/>
+      <c r="L33" s="23"/>
+      <c r="M33" s="40" t="str">
+        <v>報告書名：#{?dr_setsubi_filename_6}</v>
+      </c>
+      <c r="N33" s="41"/>
+      <c r="O33" s="41"/>
+      <c r="P33" s="41"/>
+      <c r="Q33" s="41"/>
+      <c r="R33" s="41"/>
+      <c r="S33" s="41"/>
+      <c r="T33" s="42"/>
     </row>
     <row r="34" spans="1:20" customFormat="false">
       <c r="A34" s="12"/>
-      <c r="B34" s="15"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="F34" s="80" t="s">
-        <v>45</v>
-      </c>
-      <c r="G34" s="80"/>
-      <c r="H34" s="80"/>
-      <c r="I34" s="80"/>
-      <c r="J34" s="80"/>
-      <c r="K34" s="80"/>
-      <c r="L34" s="81"/>
-      <c r="M34" s="79" t="s">
-        <v>14</v>
-      </c>
-      <c r="N34" s="80"/>
-      <c r="O34" s="80"/>
-      <c r="P34" s="80"/>
-      <c r="Q34" s="80"/>
-      <c r="R34" s="80"/>
-      <c r="S34" s="80"/>
-      <c r="T34" s="81"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="I34" s="22"/>
+      <c r="J34" s="22"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="23"/>
+      <c r="M34" s="40" t="str">
+        <v>報告書名：#{?dr_setsubi_filename_7}</v>
+      </c>
+      <c r="N34" s="41"/>
+      <c r="O34" s="41"/>
+      <c r="P34" s="41"/>
+      <c r="Q34" s="41"/>
+      <c r="R34" s="41"/>
+      <c r="S34" s="41"/>
+      <c r="T34" s="42"/>
     </row>
     <row r="35" spans="1:20" customFormat="false">
       <c r="A35" s="12"/>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="F35" s="80" t="s">
-        <v>46</v>
-      </c>
-      <c r="G35" s="80"/>
-      <c r="H35" s="80"/>
-      <c r="I35" s="80"/>
-      <c r="J35" s="80"/>
-      <c r="K35" s="80"/>
-      <c r="L35" s="81"/>
-      <c r="M35" s="79" t="s">
-        <v>111</v>
-      </c>
-      <c r="N35" s="80"/>
-      <c r="O35" s="80"/>
-      <c r="P35" s="80"/>
-      <c r="Q35" s="80"/>
-      <c r="R35" s="80"/>
-      <c r="S35" s="80"/>
-      <c r="T35" s="81"/>
-    </row>
-    <row r="36" spans="1:20" customFormat="false">
+      <c r="B35" s="16"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="F35" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="G35" s="30"/>
+      <c r="H35" s="30"/>
+      <c r="I35" s="30"/>
+      <c r="J35" s="30"/>
+      <c r="K35" s="30"/>
+      <c r="L35" s="31"/>
+      <c r="M35" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="N35" s="30"/>
+      <c r="O35" s="30"/>
+      <c r="P35" s="30"/>
+      <c r="Q35" s="30"/>
+      <c r="R35" s="30"/>
+      <c r="S35" s="30"/>
+      <c r="T35" s="31"/>
+    </row>
+    <row r="36" spans="1:21" customFormat="false">
       <c r="A36" s="12"/>
-      <c r="B36" s="15"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="F36" s="80" t="s">
-        <v>47</v>
-      </c>
-      <c r="G36" s="80"/>
-      <c r="H36" s="80"/>
-      <c r="I36" s="80"/>
-      <c r="J36" s="80"/>
-      <c r="K36" s="80"/>
-      <c r="L36" s="81"/>
-      <c r="M36" s="79" t="s">
-        <v>111</v>
-      </c>
-      <c r="N36" s="80"/>
-      <c r="O36" s="80"/>
-      <c r="P36" s="80"/>
-      <c r="Q36" s="80"/>
-      <c r="R36" s="80"/>
-      <c r="S36" s="80"/>
-      <c r="T36" s="81"/>
-    </row>
-    <row r="37" spans="1:20" customFormat="false">
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="F36" s="82" t="s">
+        <v>59</v>
+      </c>
+      <c r="G36" s="82"/>
+      <c r="H36" s="82"/>
+      <c r="I36" s="82"/>
+      <c r="J36" s="82"/>
+      <c r="K36" s="82"/>
+      <c r="L36" s="83"/>
+      <c r="M36" s="131"/>
+      <c r="N36" s="132"/>
+      <c r="O36" s="132"/>
+      <c r="P36" s="132"/>
+      <c r="Q36" s="132"/>
+      <c r="R36" s="132"/>
+      <c r="S36" s="132"/>
+      <c r="T36" s="133"/>
+      <c r="U36" s="13"/>
+    </row>
+    <row r="37" spans="1:20" customFormat="false" ht="33" customHeight="1">
       <c r="A37" s="12"/>
-      <c r="B37" s="15"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="F37" s="80" t="s">
-        <v>48</v>
-      </c>
-      <c r="G37" s="80"/>
-      <c r="H37" s="80"/>
-      <c r="I37" s="80"/>
-      <c r="J37" s="80"/>
-      <c r="K37" s="80"/>
-      <c r="L37" s="81"/>
-      <c r="M37" s="79" t="s">
-        <v>14</v>
-      </c>
-      <c r="N37" s="80"/>
-      <c r="O37" s="80"/>
-      <c r="P37" s="80"/>
-      <c r="Q37" s="80"/>
-      <c r="R37" s="80"/>
-      <c r="S37" s="80"/>
-      <c r="T37" s="81"/>
-    </row>
-    <row r="38" spans="1:20" customFormat="false">
+      <c r="B37" s="102" t="s">
+        <v>25</v>
+      </c>
+      <c r="C37" s="102"/>
+      <c r="D37" s="102"/>
+      <c r="E37" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="F37" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="G37" s="30"/>
+      <c r="H37" s="30"/>
+      <c r="I37" s="30"/>
+      <c r="J37" s="30"/>
+      <c r="K37" s="30"/>
+      <c r="L37" s="31"/>
+      <c r="M37" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="N37" s="41"/>
+      <c r="O37" s="41"/>
+      <c r="P37" s="41"/>
+      <c r="Q37" s="41"/>
+      <c r="R37" s="41"/>
+      <c r="S37" s="41"/>
+      <c r="T37" s="42"/>
+    </row>
+    <row r="38" spans="1:20" customFormat="false" ht="33" customHeight="1">
       <c r="A38" s="12"/>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>
       <c r="D38" s="15"/>
       <c r="E38" s="21" t="s">
-        <v>124</v>
+        <v>76</v>
       </c>
       <c r="F38" s="30" t="s">
-        <v>119</v>
+        <v>44</v>
       </c>
       <c r="G38" s="30"/>
       <c r="H38" s="30"/>
@@ -3318,128 +3298,128 @@
       <c r="J38" s="30"/>
       <c r="K38" s="30"/>
       <c r="L38" s="31"/>
-      <c r="M38" s="40" t="s">
-        <v>129</v>
-      </c>
-      <c r="N38" s="41"/>
-      <c r="O38" s="41"/>
-      <c r="P38" s="41"/>
-      <c r="Q38" s="41"/>
-      <c r="R38" s="41"/>
-      <c r="S38" s="41"/>
-      <c r="T38" s="42"/>
+      <c r="M38" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="N38" s="33"/>
+      <c r="O38" s="33"/>
+      <c r="P38" s="33"/>
+      <c r="Q38" s="33"/>
+      <c r="R38" s="33"/>
+      <c r="S38" s="33"/>
+      <c r="T38" s="34"/>
     </row>
     <row r="39" spans="1:20" customFormat="false">
       <c r="A39" s="12"/>
       <c r="B39" s="15"/>
       <c r="C39" s="15"/>
       <c r="D39" s="15"/>
-      <c r="E39" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="F39" s="30" t="s">
-        <v>120</v>
-      </c>
-      <c r="G39" s="30"/>
-      <c r="H39" s="30"/>
-      <c r="I39" s="30"/>
-      <c r="J39" s="30"/>
-      <c r="K39" s="30"/>
-      <c r="L39" s="31"/>
-      <c r="M39" s="40" t="s">
-        <v>130</v>
-      </c>
-      <c r="N39" s="41"/>
-      <c r="O39" s="41"/>
-      <c r="P39" s="41"/>
-      <c r="Q39" s="41"/>
-      <c r="R39" s="41"/>
-      <c r="S39" s="41"/>
-      <c r="T39" s="42"/>
+      <c r="E39" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="F39" s="80" t="s">
+        <v>45</v>
+      </c>
+      <c r="G39" s="80"/>
+      <c r="H39" s="80"/>
+      <c r="I39" s="80"/>
+      <c r="J39" s="80"/>
+      <c r="K39" s="80"/>
+      <c r="L39" s="81"/>
+      <c r="M39" s="79" t="s">
+        <v>14</v>
+      </c>
+      <c r="N39" s="80"/>
+      <c r="O39" s="80"/>
+      <c r="P39" s="80"/>
+      <c r="Q39" s="80"/>
+      <c r="R39" s="80"/>
+      <c r="S39" s="80"/>
+      <c r="T39" s="81"/>
     </row>
     <row r="40" spans="1:20" customFormat="false">
       <c r="A40" s="12"/>
       <c r="B40" s="15"/>
       <c r="C40" s="15"/>
       <c r="D40" s="15"/>
-      <c r="E40" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="F40" s="30" t="s">
-        <v>121</v>
-      </c>
-      <c r="G40" s="30"/>
-      <c r="H40" s="30"/>
-      <c r="I40" s="30"/>
-      <c r="J40" s="30"/>
-      <c r="K40" s="30"/>
-      <c r="L40" s="31"/>
-      <c r="M40" s="40" t="s">
-        <v>131</v>
-      </c>
-      <c r="N40" s="41"/>
-      <c r="O40" s="41"/>
-      <c r="P40" s="41"/>
-      <c r="Q40" s="41"/>
-      <c r="R40" s="41"/>
-      <c r="S40" s="41"/>
-      <c r="T40" s="42"/>
+      <c r="E40" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="F40" s="80" t="s">
+        <v>46</v>
+      </c>
+      <c r="G40" s="80"/>
+      <c r="H40" s="80"/>
+      <c r="I40" s="80"/>
+      <c r="J40" s="80"/>
+      <c r="K40" s="80"/>
+      <c r="L40" s="81"/>
+      <c r="M40" s="79" t="s">
+        <v>111</v>
+      </c>
+      <c r="N40" s="80"/>
+      <c r="O40" s="80"/>
+      <c r="P40" s="80"/>
+      <c r="Q40" s="80"/>
+      <c r="R40" s="80"/>
+      <c r="S40" s="80"/>
+      <c r="T40" s="81"/>
     </row>
     <row r="41" spans="1:20" customFormat="false">
       <c r="A41" s="12"/>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
       <c r="D41" s="15"/>
-      <c r="E41" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="F41" s="30" t="s">
-        <v>122</v>
-      </c>
-      <c r="G41" s="30"/>
-      <c r="H41" s="30"/>
-      <c r="I41" s="30"/>
-      <c r="J41" s="30"/>
-      <c r="K41" s="30"/>
-      <c r="L41" s="31"/>
-      <c r="M41" s="40" t="s">
-        <v>132</v>
-      </c>
-      <c r="N41" s="41"/>
-      <c r="O41" s="41"/>
-      <c r="P41" s="41"/>
-      <c r="Q41" s="41"/>
-      <c r="R41" s="41"/>
-      <c r="S41" s="41"/>
-      <c r="T41" s="42"/>
+      <c r="E41" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="F41" s="80" t="s">
+        <v>47</v>
+      </c>
+      <c r="G41" s="80"/>
+      <c r="H41" s="80"/>
+      <c r="I41" s="80"/>
+      <c r="J41" s="80"/>
+      <c r="K41" s="80"/>
+      <c r="L41" s="81"/>
+      <c r="M41" s="79" t="s">
+        <v>111</v>
+      </c>
+      <c r="N41" s="80"/>
+      <c r="O41" s="80"/>
+      <c r="P41" s="80"/>
+      <c r="Q41" s="80"/>
+      <c r="R41" s="80"/>
+      <c r="S41" s="80"/>
+      <c r="T41" s="81"/>
     </row>
     <row r="42" spans="1:20" customFormat="false">
       <c r="A42" s="12"/>
       <c r="B42" s="15"/>
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
-      <c r="E42" s="21" t="s">
-        <v>128</v>
-      </c>
-      <c r="F42" s="30" t="s">
-        <v>123</v>
-      </c>
-      <c r="G42" s="30"/>
-      <c r="H42" s="30"/>
-      <c r="I42" s="30"/>
-      <c r="J42" s="30"/>
-      <c r="K42" s="30"/>
-      <c r="L42" s="31"/>
-      <c r="M42" s="40" t="s">
-        <v>133</v>
-      </c>
-      <c r="N42" s="41"/>
-      <c r="O42" s="41"/>
-      <c r="P42" s="41"/>
-      <c r="Q42" s="41"/>
-      <c r="R42" s="41"/>
-      <c r="S42" s="41"/>
-      <c r="T42" s="42"/>
+      <c r="E42" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="F42" s="80" t="s">
+        <v>48</v>
+      </c>
+      <c r="G42" s="80"/>
+      <c r="H42" s="80"/>
+      <c r="I42" s="80"/>
+      <c r="J42" s="80"/>
+      <c r="K42" s="80"/>
+      <c r="L42" s="81"/>
+      <c r="M42" s="79" t="s">
+        <v>14</v>
+      </c>
+      <c r="N42" s="80"/>
+      <c r="O42" s="80"/>
+      <c r="P42" s="80"/>
+      <c r="Q42" s="80"/>
+      <c r="R42" s="80"/>
+      <c r="S42" s="80"/>
+      <c r="T42" s="81"/>
     </row>
     <row r="43" spans="1:20" customFormat="false">
       <c r="A43" s="12"/>
@@ -3447,10 +3427,10 @@
       <c r="C43" s="15"/>
       <c r="D43" s="15"/>
       <c r="E43" s="21" t="s">
-        <v>99</v>
+        <v>124</v>
       </c>
       <c r="F43" s="30" t="s">
-        <v>39</v>
+        <v>119</v>
       </c>
       <c r="G43" s="30"/>
       <c r="H43" s="30"/>
@@ -3458,16 +3438,16 @@
       <c r="J43" s="30"/>
       <c r="K43" s="30"/>
       <c r="L43" s="31"/>
-      <c r="M43" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="N43" s="30"/>
-      <c r="O43" s="30"/>
-      <c r="P43" s="30"/>
-      <c r="Q43" s="30"/>
-      <c r="R43" s="30"/>
-      <c r="S43" s="30"/>
-      <c r="T43" s="31"/>
+      <c r="M43" s="40" t="s">
+        <v>129</v>
+      </c>
+      <c r="N43" s="41"/>
+      <c r="O43" s="41"/>
+      <c r="P43" s="41"/>
+      <c r="Q43" s="41"/>
+      <c r="R43" s="41"/>
+      <c r="S43" s="41"/>
+      <c r="T43" s="42"/>
     </row>
     <row r="44" spans="1:20" customFormat="false">
       <c r="A44" s="12"/>
@@ -3475,10 +3455,10 @@
       <c r="C44" s="15"/>
       <c r="D44" s="15"/>
       <c r="E44" s="21" t="s">
-        <v>97</v>
+        <v>125</v>
       </c>
       <c r="F44" s="30" t="s">
-        <v>37</v>
+        <v>120</v>
       </c>
       <c r="G44" s="30"/>
       <c r="H44" s="30"/>
@@ -3486,16 +3466,16 @@
       <c r="J44" s="30"/>
       <c r="K44" s="30"/>
       <c r="L44" s="31"/>
-      <c r="M44" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="N44" s="30"/>
-      <c r="O44" s="30"/>
-      <c r="P44" s="30"/>
-      <c r="Q44" s="30"/>
-      <c r="R44" s="30"/>
-      <c r="S44" s="30"/>
-      <c r="T44" s="31"/>
+      <c r="M44" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="N44" s="41"/>
+      <c r="O44" s="41"/>
+      <c r="P44" s="41"/>
+      <c r="Q44" s="41"/>
+      <c r="R44" s="41"/>
+      <c r="S44" s="41"/>
+      <c r="T44" s="42"/>
     </row>
     <row r="45" spans="1:20" customFormat="false">
       <c r="A45" s="12"/>
@@ -3503,10 +3483,10 @@
       <c r="C45" s="15"/>
       <c r="D45" s="15"/>
       <c r="E45" s="21" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="F45" s="30" t="s">
-        <v>41</v>
+        <v>121</v>
       </c>
       <c r="G45" s="30"/>
       <c r="H45" s="30"/>
@@ -3514,16 +3494,16 @@
       <c r="J45" s="30"/>
       <c r="K45" s="30"/>
       <c r="L45" s="31"/>
-      <c r="M45" s="29" t="s">
-        <v>135</v>
-      </c>
-      <c r="N45" s="30"/>
-      <c r="O45" s="30"/>
-      <c r="P45" s="30"/>
-      <c r="Q45" s="30"/>
-      <c r="R45" s="30"/>
-      <c r="S45" s="30"/>
-      <c r="T45" s="31"/>
+      <c r="M45" s="40" t="s">
+        <v>131</v>
+      </c>
+      <c r="N45" s="41"/>
+      <c r="O45" s="41"/>
+      <c r="P45" s="41"/>
+      <c r="Q45" s="41"/>
+      <c r="R45" s="41"/>
+      <c r="S45" s="41"/>
+      <c r="T45" s="42"/>
     </row>
     <row r="46" spans="1:20" customFormat="false">
       <c r="A46" s="12"/>
@@ -3531,10 +3511,10 @@
       <c r="C46" s="15"/>
       <c r="D46" s="15"/>
       <c r="E46" s="21" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="F46" s="30" t="s">
-        <v>42</v>
+        <v>122</v>
       </c>
       <c r="G46" s="30"/>
       <c r="H46" s="30"/>
@@ -3542,16 +3522,16 @@
       <c r="J46" s="30"/>
       <c r="K46" s="30"/>
       <c r="L46" s="31"/>
-      <c r="M46" s="29" t="s">
-        <v>108</v>
-      </c>
-      <c r="N46" s="30"/>
-      <c r="O46" s="30"/>
-      <c r="P46" s="30"/>
-      <c r="Q46" s="30"/>
-      <c r="R46" s="30"/>
-      <c r="S46" s="30"/>
-      <c r="T46" s="31"/>
+      <c r="M46" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="N46" s="41"/>
+      <c r="O46" s="41"/>
+      <c r="P46" s="41"/>
+      <c r="Q46" s="41"/>
+      <c r="R46" s="41"/>
+      <c r="S46" s="41"/>
+      <c r="T46" s="42"/>
     </row>
     <row r="47" spans="1:20" customFormat="false">
       <c r="A47" s="12"/>
@@ -3559,10 +3539,10 @@
       <c r="C47" s="15"/>
       <c r="D47" s="15"/>
       <c r="E47" s="21" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="F47" s="30" t="s">
-        <v>49</v>
+        <v>123</v>
       </c>
       <c r="G47" s="30"/>
       <c r="H47" s="30"/>
@@ -3570,16 +3550,16 @@
       <c r="J47" s="30"/>
       <c r="K47" s="30"/>
       <c r="L47" s="31"/>
-      <c r="M47" s="29" t="s">
-        <v>110</v>
-      </c>
-      <c r="N47" s="30"/>
-      <c r="O47" s="30"/>
-      <c r="P47" s="30"/>
-      <c r="Q47" s="30"/>
-      <c r="R47" s="30"/>
-      <c r="S47" s="30"/>
-      <c r="T47" s="31"/>
+      <c r="M47" s="40" t="s">
+        <v>133</v>
+      </c>
+      <c r="N47" s="41"/>
+      <c r="O47" s="41"/>
+      <c r="P47" s="41"/>
+      <c r="Q47" s="41"/>
+      <c r="R47" s="41"/>
+      <c r="S47" s="41"/>
+      <c r="T47" s="42"/>
     </row>
     <row r="48" spans="1:20" customFormat="false">
       <c r="A48" s="12"/>
@@ -3587,10 +3567,10 @@
       <c r="C48" s="15"/>
       <c r="D48" s="15"/>
       <c r="E48" s="21" t="s">
-        <v>33</v>
+        <v>99</v>
       </c>
       <c r="F48" s="30" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="G48" s="30"/>
       <c r="H48" s="30"/>
@@ -3598,7 +3578,9 @@
       <c r="J48" s="30"/>
       <c r="K48" s="30"/>
       <c r="L48" s="31"/>
-      <c r="M48" s="29"/>
+      <c r="M48" s="29" t="s">
+        <v>73</v>
+      </c>
       <c r="N48" s="30"/>
       <c r="O48" s="30"/>
       <c r="P48" s="30"/>
@@ -3607,16 +3589,16 @@
       <c r="S48" s="30"/>
       <c r="T48" s="31"/>
     </row>
-    <row r="49" spans="1:20" customFormat="false" ht="33" customHeight="1">
+    <row r="49" spans="1:20" customFormat="false">
       <c r="A49" s="12"/>
       <c r="B49" s="15"/>
       <c r="C49" s="15"/>
       <c r="D49" s="15"/>
       <c r="E49" s="21" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="F49" s="30" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="G49" s="30"/>
       <c r="H49" s="30"/>
@@ -3624,16 +3606,16 @@
       <c r="J49" s="30"/>
       <c r="K49" s="30"/>
       <c r="L49" s="31"/>
-      <c r="M49" s="40" t="s">
-        <v>81</v>
-      </c>
-      <c r="N49" s="41"/>
-      <c r="O49" s="41"/>
-      <c r="P49" s="41"/>
-      <c r="Q49" s="41"/>
-      <c r="R49" s="41"/>
-      <c r="S49" s="41"/>
-      <c r="T49" s="42"/>
+      <c r="M49" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="N49" s="30"/>
+      <c r="O49" s="30"/>
+      <c r="P49" s="30"/>
+      <c r="Q49" s="30"/>
+      <c r="R49" s="30"/>
+      <c r="S49" s="30"/>
+      <c r="T49" s="31"/>
     </row>
     <row r="50" spans="1:20" customFormat="false">
       <c r="A50" s="12"/>
@@ -3641,10 +3623,10 @@
       <c r="C50" s="15"/>
       <c r="D50" s="15"/>
       <c r="E50" s="21" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F50" s="30" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="G50" s="30"/>
       <c r="H50" s="30"/>
@@ -3653,7 +3635,7 @@
       <c r="K50" s="30"/>
       <c r="L50" s="31"/>
       <c r="M50" s="29" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="N50" s="30"/>
       <c r="O50" s="30"/>
@@ -3669,10 +3651,10 @@
       <c r="C51" s="15"/>
       <c r="D51" s="15"/>
       <c r="E51" s="21" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="F51" s="30" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="G51" s="30"/>
       <c r="H51" s="30"/>
@@ -3681,7 +3663,7 @@
       <c r="K51" s="30"/>
       <c r="L51" s="31"/>
       <c r="M51" s="29" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="N51" s="30"/>
       <c r="O51" s="30"/>
@@ -3697,10 +3679,10 @@
       <c r="C52" s="15"/>
       <c r="D52" s="15"/>
       <c r="E52" s="21" t="s">
-        <v>82</v>
+        <v>109</v>
       </c>
       <c r="F52" s="30" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="G52" s="30"/>
       <c r="H52" s="30"/>
@@ -3709,7 +3691,7 @@
       <c r="K52" s="30"/>
       <c r="L52" s="31"/>
       <c r="M52" s="29" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="N52" s="30"/>
       <c r="O52" s="30"/>
@@ -3725,10 +3707,10 @@
       <c r="C53" s="15"/>
       <c r="D53" s="15"/>
       <c r="E53" s="21" t="s">
-        <v>82</v>
+        <v>33</v>
       </c>
       <c r="F53" s="30" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G53" s="30"/>
       <c r="H53" s="30"/>
@@ -3736,9 +3718,7 @@
       <c r="J53" s="30"/>
       <c r="K53" s="30"/>
       <c r="L53" s="31"/>
-      <c r="M53" s="29" t="s">
-        <v>101</v>
-      </c>
+      <c r="M53" s="29"/>
       <c r="N53" s="30"/>
       <c r="O53" s="30"/>
       <c r="P53" s="30"/>
@@ -3747,16 +3727,16 @@
       <c r="S53" s="30"/>
       <c r="T53" s="31"/>
     </row>
-    <row r="54" spans="1:20" customFormat="false">
+    <row r="54" spans="1:20" customFormat="false" ht="33" customHeight="1">
       <c r="A54" s="12"/>
       <c r="B54" s="15"/>
       <c r="C54" s="15"/>
       <c r="D54" s="15"/>
       <c r="E54" s="21" t="s">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="F54" s="30" t="s">
-        <v>138</v>
+        <v>51</v>
       </c>
       <c r="G54" s="30"/>
       <c r="H54" s="30"/>
@@ -3764,16 +3744,16 @@
       <c r="J54" s="30"/>
       <c r="K54" s="30"/>
       <c r="L54" s="31"/>
-      <c r="M54" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="N54" s="30"/>
-      <c r="O54" s="30"/>
-      <c r="P54" s="30"/>
-      <c r="Q54" s="30"/>
-      <c r="R54" s="30"/>
-      <c r="S54" s="30"/>
-      <c r="T54" s="31"/>
+      <c r="M54" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="N54" s="41"/>
+      <c r="O54" s="41"/>
+      <c r="P54" s="41"/>
+      <c r="Q54" s="41"/>
+      <c r="R54" s="41"/>
+      <c r="S54" s="41"/>
+      <c r="T54" s="42"/>
     </row>
     <row r="55" spans="1:20" customFormat="false">
       <c r="A55" s="12"/>
@@ -3781,10 +3761,10 @@
       <c r="C55" s="15"/>
       <c r="D55" s="15"/>
       <c r="E55" s="21" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="F55" s="30" t="s">
-        <v>139</v>
+        <v>52</v>
       </c>
       <c r="G55" s="30"/>
       <c r="H55" s="30"/>
@@ -3793,7 +3773,7 @@
       <c r="K55" s="30"/>
       <c r="L55" s="31"/>
       <c r="M55" s="29" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="N55" s="30"/>
       <c r="O55" s="30"/>
@@ -3809,10 +3789,10 @@
       <c r="C56" s="15"/>
       <c r="D56" s="15"/>
       <c r="E56" s="21" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="F56" s="30" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G56" s="30"/>
       <c r="H56" s="30"/>
@@ -3820,7 +3800,9 @@
       <c r="J56" s="30"/>
       <c r="K56" s="30"/>
       <c r="L56" s="31"/>
-      <c r="M56" s="29"/>
+      <c r="M56" s="29" t="s">
+        <v>65</v>
+      </c>
       <c r="N56" s="30"/>
       <c r="O56" s="30"/>
       <c r="P56" s="30"/>
@@ -3829,16 +3811,16 @@
       <c r="S56" s="30"/>
       <c r="T56" s="31"/>
     </row>
-    <row r="57" spans="1:20" customFormat="false" ht="33" customHeight="1">
+    <row r="57" spans="1:20" customFormat="false">
       <c r="A57" s="12"/>
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
       <c r="D57" s="15"/>
       <c r="E57" s="21" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="F57" s="30" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="G57" s="30"/>
       <c r="H57" s="30"/>
@@ -3846,8 +3828,8 @@
       <c r="J57" s="30"/>
       <c r="K57" s="30"/>
       <c r="L57" s="31"/>
-      <c r="M57" s="40" t="s">
-        <v>70</v>
+      <c r="M57" s="29" t="s">
+        <v>101</v>
       </c>
       <c r="N57" s="30"/>
       <c r="O57" s="30"/>
@@ -3857,16 +3839,16 @@
       <c r="S57" s="30"/>
       <c r="T57" s="31"/>
     </row>
-    <row r="58" spans="1:20" customFormat="false" ht="33" customHeight="1">
+    <row r="58" spans="1:20" customFormat="false">
       <c r="A58" s="12"/>
       <c r="B58" s="15"/>
       <c r="C58" s="15"/>
       <c r="D58" s="15"/>
       <c r="E58" s="21" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F58" s="30" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G58" s="30"/>
       <c r="H58" s="30"/>
@@ -3874,257 +3856,395 @@
       <c r="J58" s="30"/>
       <c r="K58" s="30"/>
       <c r="L58" s="31"/>
-      <c r="M58" s="32" t="s">
-        <v>77</v>
-      </c>
-      <c r="N58" s="33"/>
-      <c r="O58" s="33"/>
-      <c r="P58" s="33"/>
-      <c r="Q58" s="33"/>
-      <c r="R58" s="33"/>
-      <c r="S58" s="33"/>
-      <c r="T58" s="34"/>
+      <c r="M58" s="29" t="s">
+        <v>101</v>
+      </c>
+      <c r="N58" s="30"/>
+      <c r="O58" s="30"/>
+      <c r="P58" s="30"/>
+      <c r="Q58" s="30"/>
+      <c r="R58" s="30"/>
+      <c r="S58" s="30"/>
+      <c r="T58" s="31"/>
     </row>
     <row r="59" spans="1:20" customFormat="false">
       <c r="A59" s="12"/>
       <c r="B59" s="15"/>
       <c r="C59" s="15"/>
       <c r="D59" s="15"/>
-      <c r="E59" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="F59" s="85" t="s">
-        <v>43</v>
-      </c>
-      <c r="G59" s="85"/>
-      <c r="H59" s="85"/>
-      <c r="I59" s="85"/>
-      <c r="J59" s="85"/>
-      <c r="K59" s="85"/>
-      <c r="L59" s="86"/>
-      <c r="M59" s="84"/>
-      <c r="N59" s="85"/>
-      <c r="O59" s="85"/>
-      <c r="P59" s="85"/>
-      <c r="Q59" s="85"/>
-      <c r="R59" s="85"/>
-      <c r="S59" s="85"/>
-      <c r="T59" s="86"/>
+      <c r="E59" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="F59" s="30" t="s">
+        <v>138</v>
+      </c>
+      <c r="G59" s="30"/>
+      <c r="H59" s="30"/>
+      <c r="I59" s="30"/>
+      <c r="J59" s="30"/>
+      <c r="K59" s="30"/>
+      <c r="L59" s="31"/>
+      <c r="M59" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="N59" s="30"/>
+      <c r="O59" s="30"/>
+      <c r="P59" s="30"/>
+      <c r="Q59" s="30"/>
+      <c r="R59" s="30"/>
+      <c r="S59" s="30"/>
+      <c r="T59" s="31"/>
     </row>
     <row r="60" spans="1:20" customFormat="false">
       <c r="A60" s="12"/>
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="20" t="s">
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="F60" s="30" t="s">
+        <v>139</v>
+      </c>
+      <c r="G60" s="30"/>
+      <c r="H60" s="30"/>
+      <c r="I60" s="30"/>
+      <c r="J60" s="30"/>
+      <c r="K60" s="30"/>
+      <c r="L60" s="31"/>
+      <c r="M60" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="N60" s="30"/>
+      <c r="O60" s="30"/>
+      <c r="P60" s="30"/>
+      <c r="Q60" s="30"/>
+      <c r="R60" s="30"/>
+      <c r="S60" s="30"/>
+      <c r="T60" s="31"/>
+    </row>
+    <row r="61" spans="1:20" customFormat="false">
+      <c r="A61" s="12"/>
+      <c r="B61" s="15"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="F60" s="82" t="s">
+      <c r="F61" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="G61" s="30"/>
+      <c r="H61" s="30"/>
+      <c r="I61" s="30"/>
+      <c r="J61" s="30"/>
+      <c r="K61" s="30"/>
+      <c r="L61" s="31"/>
+      <c r="M61" s="29"/>
+      <c r="N61" s="30"/>
+      <c r="O61" s="30"/>
+      <c r="P61" s="30"/>
+      <c r="Q61" s="30"/>
+      <c r="R61" s="30"/>
+      <c r="S61" s="30"/>
+      <c r="T61" s="31"/>
+    </row>
+    <row r="62" spans="1:20" customFormat="false" ht="33" customHeight="1">
+      <c r="A62" s="12"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="15"/>
+      <c r="E62" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="F62" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="G62" s="30"/>
+      <c r="H62" s="30"/>
+      <c r="I62" s="30"/>
+      <c r="J62" s="30"/>
+      <c r="K62" s="30"/>
+      <c r="L62" s="31"/>
+      <c r="M62" s="40" t="s">
+        <v>70</v>
+      </c>
+      <c r="N62" s="30"/>
+      <c r="O62" s="30"/>
+      <c r="P62" s="30"/>
+      <c r="Q62" s="30"/>
+      <c r="R62" s="30"/>
+      <c r="S62" s="30"/>
+      <c r="T62" s="31"/>
+    </row>
+    <row r="63" spans="1:20" customFormat="false" ht="33" customHeight="1">
+      <c r="A63" s="12"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="15"/>
+      <c r="E63" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="F63" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="G63" s="30"/>
+      <c r="H63" s="30"/>
+      <c r="I63" s="30"/>
+      <c r="J63" s="30"/>
+      <c r="K63" s="30"/>
+      <c r="L63" s="31"/>
+      <c r="M63" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="N63" s="33"/>
+      <c r="O63" s="33"/>
+      <c r="P63" s="33"/>
+      <c r="Q63" s="33"/>
+      <c r="R63" s="33"/>
+      <c r="S63" s="33"/>
+      <c r="T63" s="34"/>
+    </row>
+    <row r="64" spans="1:20" customFormat="false">
+      <c r="A64" s="12"/>
+      <c r="B64" s="15"/>
+      <c r="C64" s="15"/>
+      <c r="D64" s="15"/>
+      <c r="E64" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="F64" s="85" t="s">
+        <v>43</v>
+      </c>
+      <c r="G64" s="85"/>
+      <c r="H64" s="85"/>
+      <c r="I64" s="85"/>
+      <c r="J64" s="85"/>
+      <c r="K64" s="85"/>
+      <c r="L64" s="86"/>
+      <c r="M64" s="84"/>
+      <c r="N64" s="85"/>
+      <c r="O64" s="85"/>
+      <c r="P64" s="85"/>
+      <c r="Q64" s="85"/>
+      <c r="R64" s="85"/>
+      <c r="S64" s="85"/>
+      <c r="T64" s="86"/>
+    </row>
+    <row r="65" spans="1:20" customFormat="false">
+      <c r="A65" s="12"/>
+      <c r="B65" s="14"/>
+      <c r="C65" s="14"/>
+      <c r="D65" s="14"/>
+      <c r="E65" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="F65" s="82" t="s">
         <v>58</v>
       </c>
-      <c r="G60" s="82"/>
-      <c r="H60" s="82"/>
-      <c r="I60" s="82"/>
-      <c r="J60" s="82"/>
-      <c r="K60" s="82"/>
-      <c r="L60" s="83"/>
-      <c r="M60" s="84"/>
-      <c r="N60" s="85"/>
-      <c r="O60" s="85"/>
-      <c r="P60" s="85"/>
-      <c r="Q60" s="85"/>
-      <c r="R60" s="85"/>
-      <c r="S60" s="85"/>
-      <c r="T60" s="86"/>
-    </row>
-    <row r="61" spans="1:20" customFormat="false">
-      <c r="A61" s="96" t="s">
+      <c r="G65" s="82"/>
+      <c r="H65" s="82"/>
+      <c r="I65" s="82"/>
+      <c r="J65" s="82"/>
+      <c r="K65" s="82"/>
+      <c r="L65" s="83"/>
+      <c r="M65" s="84"/>
+      <c r="N65" s="85"/>
+      <c r="O65" s="85"/>
+      <c r="P65" s="85"/>
+      <c r="Q65" s="85"/>
+      <c r="R65" s="85"/>
+      <c r="S65" s="85"/>
+      <c r="T65" s="86"/>
+    </row>
+    <row r="66" spans="1:20" customFormat="false">
+      <c r="A66" s="96" t="s">
         <v>26</v>
       </c>
-      <c r="B61" s="97"/>
-      <c r="C61" s="87" t="s">
+      <c r="B66" s="97"/>
+      <c r="C66" s="87" t="s">
         <v>22</v>
       </c>
-      <c r="D61" s="88"/>
-      <c r="E61" s="88"/>
-      <c r="F61" s="89"/>
-      <c r="G61" s="87" t="s">
+      <c r="D66" s="88"/>
+      <c r="E66" s="88"/>
+      <c r="F66" s="89"/>
+      <c r="G66" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="H61" s="88"/>
-      <c r="I61" s="88"/>
-      <c r="J61" s="89"/>
-      <c r="K61" s="87" t="s">
+      <c r="H66" s="88"/>
+      <c r="I66" s="88"/>
+      <c r="J66" s="89"/>
+      <c r="K66" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="L61" s="88"/>
-      <c r="M61" s="88"/>
-      <c r="N61" s="89"/>
-      <c r="O61" s="87" t="s">
+      <c r="L66" s="88"/>
+      <c r="M66" s="88"/>
+      <c r="N66" s="89"/>
+      <c r="O66" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="P61" s="88"/>
-      <c r="Q61" s="88"/>
-      <c r="R61" s="88"/>
-      <c r="S61" s="88"/>
-      <c r="T61" s="89"/>
-    </row>
-    <row r="62" spans="1:20" customFormat="false">
-      <c r="A62" s="98"/>
-      <c r="B62" s="99"/>
-      <c r="C62" s="92" t="s">
+      <c r="P66" s="88"/>
+      <c r="Q66" s="88"/>
+      <c r="R66" s="88"/>
+      <c r="S66" s="88"/>
+      <c r="T66" s="89"/>
+    </row>
+    <row r="67" spans="1:20" customFormat="false">
+      <c r="A67" s="98"/>
+      <c r="B67" s="99"/>
+      <c r="C67" s="92" t="s">
         <v>29</v>
       </c>
-      <c r="D62" s="92"/>
-      <c r="E62" s="92" t="s">
+      <c r="D67" s="92"/>
+      <c r="E67" s="92" t="s">
         <v>30</v>
       </c>
-      <c r="F62" s="92"/>
-      <c r="G62" s="92" t="s">
+      <c r="F67" s="92"/>
+      <c r="G67" s="92" t="s">
         <v>29</v>
       </c>
-      <c r="H62" s="92"/>
-      <c r="I62" s="92" t="s">
+      <c r="H67" s="92"/>
+      <c r="I67" s="92" t="s">
         <v>30</v>
       </c>
-      <c r="J62" s="92"/>
-      <c r="K62" s="92" t="s">
+      <c r="J67" s="92"/>
+      <c r="K67" s="92" t="s">
         <v>29</v>
       </c>
-      <c r="L62" s="92"/>
-      <c r="M62" s="92" t="s">
+      <c r="L67" s="92"/>
+      <c r="M67" s="92" t="s">
         <v>30</v>
       </c>
-      <c r="N62" s="92"/>
-      <c r="O62" s="92" t="s">
+      <c r="N67" s="92"/>
+      <c r="O67" s="92" t="s">
         <v>29</v>
       </c>
-      <c r="P62" s="92"/>
-      <c r="Q62" s="90"/>
-      <c r="R62" s="91"/>
-      <c r="S62" s="90"/>
-      <c r="T62" s="91"/>
-    </row>
-    <row r="63" spans="1:20" customFormat="false">
-      <c r="A63" s="3" t="s">
+      <c r="P67" s="92"/>
+      <c r="Q67" s="90"/>
+      <c r="R67" s="91"/>
+      <c r="S67" s="90"/>
+      <c r="T67" s="91"/>
+    </row>
+    <row r="68" spans="1:20" customFormat="false">
+      <c r="A68" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B63" s="4"/>
-      <c r="C63" s="93" t="s">
+      <c r="B68" s="4"/>
+      <c r="C68" s="93" t="s">
         <v>93</v>
       </c>
-      <c r="D63" s="94"/>
-      <c r="E63" s="93" t="s">
+      <c r="D68" s="94"/>
+      <c r="E68" s="93" t="s">
         <v>94</v>
       </c>
-      <c r="F63" s="94"/>
-      <c r="G63" s="93" t="s">
+      <c r="F68" s="94"/>
+      <c r="G68" s="93" t="s">
         <v>85</v>
       </c>
-      <c r="H63" s="94"/>
-      <c r="I63" s="93" t="s">
+      <c r="H68" s="94"/>
+      <c r="I68" s="93" t="s">
         <v>86</v>
       </c>
-      <c r="J63" s="94"/>
-      <c r="K63" s="95" t="s">
+      <c r="J68" s="94"/>
+      <c r="K68" s="95" t="s">
         <v>91</v>
       </c>
-      <c r="L63" s="94"/>
-      <c r="M63" s="95" t="s">
+      <c r="L68" s="94"/>
+      <c r="M68" s="95" t="s">
         <v>89</v>
       </c>
-      <c r="N63" s="94"/>
-      <c r="O63" s="35"/>
-      <c r="P63" s="36"/>
-      <c r="Q63" s="27"/>
-      <c r="R63" s="28"/>
-      <c r="S63" s="27"/>
-      <c r="T63" s="27"/>
-    </row>
-    <row r="64" spans="1:20" customFormat="false">
-      <c r="A64" s="5" t="s">
+      <c r="N68" s="94"/>
+      <c r="O68" s="35"/>
+      <c r="P68" s="36"/>
+      <c r="Q68" s="27"/>
+      <c r="R68" s="28"/>
+      <c r="S68" s="27"/>
+      <c r="T68" s="27"/>
+    </row>
+    <row r="69" spans="1:20" customFormat="false">
+      <c r="A69" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B64" s="6"/>
-      <c r="C64" s="35"/>
-      <c r="D64" s="35"/>
-      <c r="E64" s="35"/>
-      <c r="F64" s="35"/>
-      <c r="G64" s="35"/>
-      <c r="H64" s="35"/>
-      <c r="I64" s="35"/>
-      <c r="J64" s="35"/>
-      <c r="K64" s="35"/>
-      <c r="L64" s="35"/>
-      <c r="M64" s="35"/>
-      <c r="N64" s="35"/>
-      <c r="O64" s="35"/>
-      <c r="P64" s="36"/>
-      <c r="Q64" s="27"/>
-      <c r="R64" s="28"/>
-      <c r="S64" s="27"/>
-      <c r="T64" s="28"/>
-    </row>
-    <row r="65" spans="1:20" customFormat="false">
-      <c r="A65" s="9" t="s">
+      <c r="B69" s="6"/>
+      <c r="C69" s="35"/>
+      <c r="D69" s="35"/>
+      <c r="E69" s="35"/>
+      <c r="F69" s="35"/>
+      <c r="G69" s="35"/>
+      <c r="H69" s="35"/>
+      <c r="I69" s="35"/>
+      <c r="J69" s="35"/>
+      <c r="K69" s="35"/>
+      <c r="L69" s="35"/>
+      <c r="M69" s="35"/>
+      <c r="N69" s="35"/>
+      <c r="O69" s="35"/>
+      <c r="P69" s="36"/>
+      <c r="Q69" s="27"/>
+      <c r="R69" s="28"/>
+      <c r="S69" s="27"/>
+      <c r="T69" s="28"/>
+    </row>
+    <row r="70" spans="1:20" customFormat="false">
+      <c r="A70" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B65" s="10"/>
-      <c r="C65" s="93" t="s">
+      <c r="B70" s="10"/>
+      <c r="C70" s="93" t="s">
         <v>95</v>
       </c>
-      <c r="D65" s="94"/>
-      <c r="E65" s="93" t="s">
+      <c r="D70" s="94"/>
+      <c r="E70" s="93" t="s">
         <v>96</v>
       </c>
-      <c r="F65" s="94"/>
-      <c r="G65" s="93" t="s">
+      <c r="F70" s="94"/>
+      <c r="G70" s="93" t="s">
         <v>87</v>
       </c>
-      <c r="H65" s="94"/>
-      <c r="I65" s="93" t="s">
+      <c r="H70" s="94"/>
+      <c r="I70" s="93" t="s">
         <v>88</v>
       </c>
-      <c r="J65" s="94"/>
-      <c r="K65" s="95" t="s">
+      <c r="J70" s="94"/>
+      <c r="K70" s="95" t="s">
         <v>92</v>
       </c>
-      <c r="L65" s="94"/>
-      <c r="M65" s="95" t="s">
+      <c r="L70" s="94"/>
+      <c r="M70" s="95" t="s">
         <v>90</v>
       </c>
-      <c r="N65" s="94"/>
-      <c r="O65" s="35"/>
-      <c r="P65" s="36"/>
-      <c r="Q65" s="27"/>
-      <c r="R65" s="28"/>
-      <c r="S65" s="27"/>
-      <c r="T65" s="28"/>
+      <c r="N70" s="94"/>
+      <c r="O70" s="35"/>
+      <c r="P70" s="36"/>
+      <c r="Q70" s="27"/>
+      <c r="R70" s="28"/>
+      <c r="S70" s="27"/>
+      <c r="T70" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="167">
+  <mergeCells count="172">
     <mergeCell ref="M25:T25"/>
     <mergeCell ref="M26:T26"/>
-    <mergeCell ref="M30:T30"/>
-    <mergeCell ref="M31:T31"/>
-    <mergeCell ref="M46:T46"/>
+    <mergeCell ref="M35:T35"/>
+    <mergeCell ref="M36:T36"/>
+    <mergeCell ref="M51:T51"/>
+    <mergeCell ref="F49:L49"/>
+    <mergeCell ref="F50:L50"/>
+    <mergeCell ref="M43:T43"/>
+    <mergeCell ref="M48:T48"/>
+    <mergeCell ref="M49:T49"/>
+    <mergeCell ref="M50:T50"/>
+    <mergeCell ref="M38:T38"/>
+    <mergeCell ref="M40:T40"/>
+    <mergeCell ref="M27:T27"/>
     <mergeCell ref="F44:L44"/>
     <mergeCell ref="F45:L45"/>
-    <mergeCell ref="M38:T38"/>
-    <mergeCell ref="M43:T43"/>
+    <mergeCell ref="F46:L46"/>
+    <mergeCell ref="F47:L47"/>
     <mergeCell ref="M44:T44"/>
     <mergeCell ref="M45:T45"/>
-    <mergeCell ref="M33:T33"/>
-    <mergeCell ref="M35:T35"/>
-    <mergeCell ref="M27:T27"/>
-    <mergeCell ref="F39:L39"/>
-    <mergeCell ref="F40:L40"/>
-    <mergeCell ref="F41:L41"/>
-    <mergeCell ref="F42:L42"/>
-    <mergeCell ref="M39:T39"/>
-    <mergeCell ref="M40:T40"/>
-    <mergeCell ref="M41:T41"/>
-    <mergeCell ref="M42:T42"/>
+    <mergeCell ref="M46:T46"/>
+    <mergeCell ref="M47:T47"/>
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="C5:T5"/>
     <mergeCell ref="A8:B8"/>
@@ -4149,80 +4269,80 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A11:D18"/>
     <mergeCell ref="C2:T2"/>
-    <mergeCell ref="A61:B62"/>
-    <mergeCell ref="C61:F61"/>
+    <mergeCell ref="A66:B67"/>
+    <mergeCell ref="C66:F66"/>
     <mergeCell ref="F20:L20"/>
     <mergeCell ref="F23:L23"/>
     <mergeCell ref="F24:L24"/>
     <mergeCell ref="F25:L25"/>
     <mergeCell ref="F26:L26"/>
-    <mergeCell ref="F30:L30"/>
-    <mergeCell ref="F46:L46"/>
-    <mergeCell ref="F47:L47"/>
-    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="F35:L35"/>
+    <mergeCell ref="F51:L51"/>
+    <mergeCell ref="F52:L52"/>
+    <mergeCell ref="B37:D37"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="F27:L27"/>
-    <mergeCell ref="F38:L38"/>
     <mergeCell ref="F43:L43"/>
-    <mergeCell ref="F34:L34"/>
-    <mergeCell ref="F35:L35"/>
+    <mergeCell ref="F48:L48"/>
+    <mergeCell ref="F39:L39"/>
+    <mergeCell ref="F40:L40"/>
+    <mergeCell ref="F41:L41"/>
+    <mergeCell ref="F42:L42"/>
+    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="E67:F67"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="I67:J67"/>
+    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="E69:F69"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="I69:J69"/>
+    <mergeCell ref="O70:P70"/>
+    <mergeCell ref="C68:D68"/>
+    <mergeCell ref="E68:F68"/>
+    <mergeCell ref="I68:J68"/>
+    <mergeCell ref="K68:L68"/>
+    <mergeCell ref="M68:N68"/>
+    <mergeCell ref="G68:H68"/>
+    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="I70:J70"/>
+    <mergeCell ref="K70:L70"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="C70:D70"/>
+    <mergeCell ref="M70:N70"/>
+    <mergeCell ref="M65:T65"/>
+    <mergeCell ref="M57:T57"/>
+    <mergeCell ref="F62:L62"/>
+    <mergeCell ref="M62:T62"/>
+    <mergeCell ref="G66:J66"/>
+    <mergeCell ref="K66:N66"/>
+    <mergeCell ref="O66:T66"/>
+    <mergeCell ref="S68:T68"/>
+    <mergeCell ref="Q68:R68"/>
+    <mergeCell ref="M64:T64"/>
+    <mergeCell ref="F64:L64"/>
+    <mergeCell ref="Q67:R67"/>
+    <mergeCell ref="S67:T67"/>
+    <mergeCell ref="K67:L67"/>
+    <mergeCell ref="M67:N67"/>
+    <mergeCell ref="O67:P67"/>
+    <mergeCell ref="F65:L65"/>
+    <mergeCell ref="M52:T52"/>
+    <mergeCell ref="M28:T28"/>
+    <mergeCell ref="M37:T37"/>
+    <mergeCell ref="F63:L63"/>
+    <mergeCell ref="F57:L57"/>
+    <mergeCell ref="F58:L58"/>
+    <mergeCell ref="F59:L59"/>
+    <mergeCell ref="F61:L61"/>
+    <mergeCell ref="M42:T42"/>
+    <mergeCell ref="M39:T39"/>
+    <mergeCell ref="M41:T41"/>
     <mergeCell ref="F36:L36"/>
     <mergeCell ref="F37:L37"/>
-    <mergeCell ref="C62:D62"/>
-    <mergeCell ref="E62:F62"/>
-    <mergeCell ref="G62:H62"/>
-    <mergeCell ref="I62:J62"/>
-    <mergeCell ref="C64:D64"/>
-    <mergeCell ref="E64:F64"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="I64:J64"/>
-    <mergeCell ref="O65:P65"/>
-    <mergeCell ref="C63:D63"/>
-    <mergeCell ref="E63:F63"/>
-    <mergeCell ref="I63:J63"/>
-    <mergeCell ref="K63:L63"/>
-    <mergeCell ref="M63:N63"/>
-    <mergeCell ref="G63:H63"/>
-    <mergeCell ref="E65:F65"/>
-    <mergeCell ref="I65:J65"/>
-    <mergeCell ref="K65:L65"/>
-    <mergeCell ref="G65:H65"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="F38:L38"/>
+    <mergeCell ref="F60:L60"/>
     <mergeCell ref="M60:T60"/>
-    <mergeCell ref="M52:T52"/>
-    <mergeCell ref="F57:L57"/>
-    <mergeCell ref="M57:T57"/>
-    <mergeCell ref="G61:J61"/>
-    <mergeCell ref="K61:N61"/>
-    <mergeCell ref="O61:T61"/>
-    <mergeCell ref="S63:T63"/>
-    <mergeCell ref="Q63:R63"/>
-    <mergeCell ref="M59:T59"/>
-    <mergeCell ref="F59:L59"/>
-    <mergeCell ref="Q62:R62"/>
-    <mergeCell ref="S62:T62"/>
-    <mergeCell ref="K62:L62"/>
-    <mergeCell ref="M62:N62"/>
-    <mergeCell ref="O62:P62"/>
-    <mergeCell ref="F60:L60"/>
-    <mergeCell ref="M47:T47"/>
-    <mergeCell ref="M28:T28"/>
-    <mergeCell ref="M32:T32"/>
-    <mergeCell ref="F58:L58"/>
-    <mergeCell ref="F52:L52"/>
-    <mergeCell ref="F53:L53"/>
-    <mergeCell ref="F54:L54"/>
-    <mergeCell ref="F56:L56"/>
-    <mergeCell ref="M37:T37"/>
-    <mergeCell ref="M34:T34"/>
-    <mergeCell ref="M36:T36"/>
-    <mergeCell ref="F31:L31"/>
-    <mergeCell ref="F32:L32"/>
-    <mergeCell ref="F33:L33"/>
-    <mergeCell ref="F55:L55"/>
-    <mergeCell ref="M55:T55"/>
     <mergeCell ref="C3:T3"/>
     <mergeCell ref="C4:T4"/>
     <mergeCell ref="C6:T6"/>
@@ -4245,31 +4365,36 @@
     <mergeCell ref="J7:M7"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="Q65:R65"/>
-    <mergeCell ref="S65:T65"/>
+    <mergeCell ref="Q70:R70"/>
+    <mergeCell ref="S70:T70"/>
+    <mergeCell ref="M58:T58"/>
+    <mergeCell ref="M59:T59"/>
+    <mergeCell ref="M61:T61"/>
+    <mergeCell ref="M63:T63"/>
+    <mergeCell ref="M56:T56"/>
+    <mergeCell ref="O68:P68"/>
+    <mergeCell ref="M23:T23"/>
+    <mergeCell ref="M24:T24"/>
+    <mergeCell ref="K69:L69"/>
+    <mergeCell ref="M69:N69"/>
+    <mergeCell ref="O69:P69"/>
+    <mergeCell ref="Q69:R69"/>
+    <mergeCell ref="S69:T69"/>
+    <mergeCell ref="F53:L53"/>
+    <mergeCell ref="F54:L54"/>
+    <mergeCell ref="F55:L55"/>
+    <mergeCell ref="F56:L56"/>
+    <mergeCell ref="M55:T55"/>
     <mergeCell ref="M53:T53"/>
     <mergeCell ref="M54:T54"/>
-    <mergeCell ref="M56:T56"/>
-    <mergeCell ref="M58:T58"/>
-    <mergeCell ref="M51:T51"/>
-    <mergeCell ref="O63:P63"/>
-    <mergeCell ref="M23:T23"/>
-    <mergeCell ref="M24:T24"/>
-    <mergeCell ref="K64:L64"/>
-    <mergeCell ref="M64:N64"/>
-    <mergeCell ref="O64:P64"/>
-    <mergeCell ref="Q64:R64"/>
-    <mergeCell ref="S64:T64"/>
-    <mergeCell ref="F48:L48"/>
-    <mergeCell ref="F49:L49"/>
-    <mergeCell ref="F50:L50"/>
-    <mergeCell ref="F51:L51"/>
-    <mergeCell ref="M50:T50"/>
-    <mergeCell ref="M48:T48"/>
-    <mergeCell ref="M49:T49"/>
     <mergeCell ref="M29:T29"/>
-    <mergeCell ref="F28:L29"/>
-    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="M30:T30"/>
+    <mergeCell ref="M31:T31"/>
+    <mergeCell ref="M32:T32"/>
+    <mergeCell ref="M33:T33"/>
+    <mergeCell ref="M34:T34"/>
+    <mergeCell ref="F28:L34"/>
+    <mergeCell ref="E28:E34"/>
   </mergeCells>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7086614173228347" right="0.7086614173228347" top="0" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>